<commit_message>
SCRUM-56: TCs_Decision + update cac file
</commit_message>
<xml_diff>
--- a/Docs/QA-Testing/Bug_Report.xlsx
+++ b/Docs/QA-Testing/Bug_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\MouseWithoutBorders\repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C89017-BF22-40C9-B3F0-8C12DE266735}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5563064C-682F-4D49-9677-CE2D127AAFF0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23490" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="107">
   <si>
     <t>Bug ID</t>
   </si>
@@ -321,13 +321,36 @@
   </si>
   <si>
     <t>TC_FE_EMP_09, TC_FE_MRG_09</t>
+  </si>
+  <si>
+    <t>[API][Security] Hệ thống cho phép đăng ký với role tùy ý (Privilege Escalation)</t>
+  </si>
+  <si>
+    <t>SCRUM-58</t>
+  </si>
+  <si>
+    <t>TC-SEC-01</t>
+  </si>
+  <si>
+    <t>1. POST /register với body chứa role = "ROLE_MANAGER" 
+2. Đăng nhập tài khoản vừa tạo 
+3. Kiểm tra quyền Manager</t>
+  </si>
+  <si>
+    <t>Luôn gán ROLE_CUSTOMER, bỏ qua giá trị client gửi</t>
+  </si>
+  <si>
+    <t>Lưu đúng role client gửi (ROLE_MANAGER) → leo thang đặc quyền</t>
+  </si>
+  <si>
+    <t>Root cause: UserController.save() thiếu dòng user.setRole("ROLE_CUSTOMER").</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -362,6 +385,11 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -435,7 +463,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -449,6 +477,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -756,16 +787,17 @@
   <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" customWidth="1"/>
     <col min="2" max="2" width="30.42578125" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="36" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
-    <col min="8" max="10" width="12" customWidth="1"/>
+    <col min="8" max="8" width="15.140625" customWidth="1"/>
+    <col min="9" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="12" max="12" width="39.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -912,7 +944,7 @@
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
     </row>
-    <row r="5" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>59</v>
       </c>
@@ -1162,33 +1194,55 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
+    <row r="12" spans="1:12" ht="63" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K12" s="7"/>
+      <c r="L12" s="6" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="13" spans="1:12" ht="165" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
     </row>
     <row r="14" spans="1:12" ht="181.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>

</xml_diff>

<commit_message>
SCRUM-57: Tích hợp SRS, RTM, Test Plan và State Transition Decision Table
</commit_message>
<xml_diff>
--- a/Docs/QA-Testing/Bug_Report.xlsx
+++ b/Docs/QA-Testing/Bug_Report.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\MouseWithoutBorders\repo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\MouseWithoutBorders\sp3\dasua\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5563064C-682F-4D49-9677-CE2D127AAFF0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F82BC46-2467-4FB0-A98F-2633A994D86B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23490" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10200" windowHeight="7560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="115">
   <si>
     <t>Bug ID</t>
   </si>
@@ -344,6 +344,33 @@
   </si>
   <si>
     <t>Root cause: UserController.save() thiếu dòng user.setRole("ROLE_CUSTOMER").</t>
+  </si>
+  <si>
+    <t>SCRUM-59</t>
+  </si>
+  <si>
+    <t>PATCH /order/cancel/{id}
+PATCH /order/finish/{id}</t>
+  </si>
+  <si>
+    <t>TC-ST-03, TC-ST-04, TC-ST-05</t>
+  </si>
+  <si>
+    <t>1. Lấy đơn hàng đã ở trạng thái CANCELED hoặc FINISHED
+2. Gọi API Cancel hoặc Finish trên đơn đó
+3. Quan sát response</t>
+  </si>
+  <si>
+    <t>Trả về 400 Bad Request hoặc 409 Conflict</t>
+  </si>
+  <si>
+    <t>Trả về 500 Internal Server Error + message "Status is not correct"</t>
+  </si>
+  <si>
+    <t>Phát hiện từ State Transition Testing. Hệ thống có chặn nhưng xử lý exception sai.</t>
+  </si>
+  <si>
+    <t>[API][Order] Invalid status transition trả về 500 thay vì 4xx</t>
   </si>
 </sst>
 </file>
@@ -375,23 +402,25 @@
       <family val="1"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <sz val="13"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
     </font>
     <font>
-      <sz val="12"/>
+      <b/>
+      <sz val="13"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="163"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="13"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="163"/>
     </font>
   </fonts>
   <fills count="3">
@@ -408,27 +437,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB0B0B0"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB0B0B0"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB0B0B0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB0B0B0"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -463,23 +477,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -800,449 +811,471 @@
     <col min="12" max="12" width="39.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:12" ht="33" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="1:12" ht="66" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6" t="s">
+      <c r="K2" s="5"/>
+      <c r="L2" s="5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:12" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6" t="s">
+      <c r="K3" s="5"/>
+      <c r="L3" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    <row r="4" spans="1:12" ht="66" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
     </row>
     <row r="5" spans="1:12" ht="54" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6" t="s">
+      <c r="K5" s="5"/>
+      <c r="L5" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:12" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6" t="s">
+      <c r="K6" s="5"/>
+      <c r="L6" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:12" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="5">
         <v>400</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6" t="s">
+      <c r="K7" s="5"/>
+      <c r="L7" s="5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:12" ht="33" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="5">
         <v>500</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J8" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6" t="s">
+      <c r="K8" s="5"/>
+      <c r="L8" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+    <row r="9" spans="1:12" ht="33" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="5">
         <v>400</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="5">
         <v>500</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-    </row>
-    <row r="10" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+    </row>
+    <row r="10" spans="1:12" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="5">
         <v>400</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="I10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J10" s="6" t="s">
+      <c r="J10" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6" t="s">
+      <c r="K10" s="5"/>
+      <c r="L10" s="5" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="63" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:12" ht="66" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="I11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J11" s="6" t="s">
+      <c r="J11" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6" t="s">
+      <c r="K11" s="5"/>
+      <c r="L11" s="5" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="63" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+    <row r="12" spans="1:12" ht="66" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="I12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J12" s="6" t="s">
+      <c r="J12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="K12" s="7"/>
-      <c r="L12" s="6" t="s">
+      <c r="K12" s="6"/>
+      <c r="L12" s="5" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="165" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
+    <row r="13" spans="1:12" ht="82.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="K13" s="6"/>
+      <c r="L13" s="5" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="14" spans="1:12" ht="181.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>

</xml_diff>

<commit_message>
SCRUM-60: hoàn thiện Register (Standard BVA 21 TC + Robusness
</commit_message>
<xml_diff>
--- a/Docs/QA-Testing/Bug_Report.xlsx
+++ b/Docs/QA-Testing/Bug_Report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20398"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\MouseWithoutBorders\sp3\dasua\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\task1sp4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F82BC46-2467-4FB0-A98F-2633A994D86B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{104A9A42-FF6E-4012-B16A-ADD71FA9CC5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10200" windowHeight="7560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="124">
   <si>
     <t>Bug ID</t>
   </si>
@@ -371,6 +371,33 @@
   </si>
   <si>
     <t>[API][Order] Invalid status transition trả về 500 thay vì 4xx</t>
+  </si>
+  <si>
+    <t>SCRUM-66</t>
+  </si>
+  <si>
+    <t>SCRUM-67</t>
+  </si>
+  <si>
+    <t>SCRUM-68</t>
+  </si>
+  <si>
+    <t>[API][User] Hệ thống chấp nhận đăng ký với email 5 ký tự</t>
+  </si>
+  <si>
+    <t>[API][User] Hệ thống chấp nhận đăng ký với mật khẩu 21 ký tự</t>
+  </si>
+  <si>
+    <t>TC-REG-ROB-02</t>
+  </si>
+  <si>
+    <t>TC-REG-ROB-03</t>
+  </si>
+  <si>
+    <t>TC-REG-ROB-04</t>
+  </si>
+  <si>
+    <t>[API][User] Hệ thống chấp nhận đăng ký tài khoản với email dài hơn 50 ký tự (51 ký tự)</t>
   </si>
 </sst>
 </file>
@@ -402,10 +429,10 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="13"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="163"/>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -413,14 +440,12 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-      <charset val="163"/>
     </font>
     <font>
       <sz val="13"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-      <charset val="163"/>
     </font>
   </fonts>
   <fills count="3">
@@ -437,7 +462,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -460,38 +485,28 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB0B0B0"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB0B0B0"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFB0B0B0"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -795,588 +810,671 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" customWidth="1"/>
+    <col min="1" max="1" width="14.88671875" customWidth="1"/>
+    <col min="2" max="2" width="30.44140625" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" customWidth="1"/>
     <col min="5" max="5" width="36" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" customWidth="1"/>
+    <col min="8" max="8" width="15.109375" customWidth="1"/>
     <col min="9" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="39.42578125" customWidth="1"/>
+    <col min="12" max="12" width="39.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="33" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:12" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="66" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:12" ht="67.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5" t="s">
+      <c r="K2" s="4"/>
+      <c r="L2" s="4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5" t="s">
+      <c r="K3" s="4"/>
+      <c r="L3" s="4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="66" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:12" ht="67.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J4" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-    </row>
-    <row r="5" spans="1:12" ht="54" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+    </row>
+    <row r="5" spans="1:12" ht="54" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5" t="s">
+      <c r="K5" s="4"/>
+      <c r="L5" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="J6" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5" t="s">
+      <c r="K6" s="4"/>
+      <c r="L6" s="4" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="4">
         <v>400</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5" t="s">
+      <c r="K7" s="4"/>
+      <c r="L7" s="4" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="33" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+    <row r="8" spans="1:12" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="4">
         <v>500</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5" t="s">
+      <c r="K8" s="4"/>
+      <c r="L8" s="4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="33" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:12" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="4">
         <v>400</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="4">
         <v>500</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-    </row>
-    <row r="10" spans="1:12" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+    </row>
+    <row r="10" spans="1:12" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="4">
         <v>400</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="J10" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5" t="s">
+      <c r="K10" s="4"/>
+      <c r="L10" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="66" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+    <row r="11" spans="1:12" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G11" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="J11" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5" t="s">
+      <c r="K11" s="4"/>
+      <c r="L11" s="4" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="66" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+    <row r="12" spans="1:12" ht="67.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="H12" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="I12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J12" s="5" t="s">
+      <c r="J12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="K12" s="6"/>
-      <c r="L12" s="5" t="s">
+      <c r="K12" s="5"/>
+      <c r="L12" s="4" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="82.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+    <row r="13" spans="1:12" ht="84" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="J13" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="K13" s="6"/>
-      <c r="L13" s="5" t="s">
+      <c r="K13" s="5"/>
+      <c r="L13" s="4" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="181.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
+    <row r="14" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E14" s="5"/>
+      <c r="F14" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+    </row>
+    <row r="15" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="E15" s="4"/>
+      <c r="F15" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+    </row>
+    <row r="16" spans="1:12" ht="67.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E16" s="4"/>
+      <c r="F16" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>41</v>
       </c>

</xml_diff>

<commit_message>
SCRUM-76: Fix product price and stock validation
</commit_message>
<xml_diff>
--- a/Docs/QA-Testing/Bug_Report.xlsx
+++ b/Docs/QA-Testing/Bug_Report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20398"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\MouseWithoutBorders\sss\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KCPM - NAM3\Online-Store\Docs\QA-Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{063C68EA-83AA-456F-B6FC-1FE32F3E45D8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D3D338-CF33-4BDB-8983-33F4CECBC325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="144">
   <si>
     <t>Bug ID</t>
   </si>
@@ -868,22 +868,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L20"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" customWidth="1"/>
+    <col min="1" max="1" width="14.88671875" customWidth="1"/>
+    <col min="2" max="2" width="30.44140625" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="22.42578125" customWidth="1"/>
+    <col min="4" max="4" width="22.44140625" customWidth="1"/>
     <col min="5" max="5" width="36" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" customWidth="1"/>
+    <col min="8" max="8" width="15.109375" customWidth="1"/>
     <col min="9" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="39.42578125" customWidth="1"/>
+    <col min="12" max="12" width="39.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -921,7 +921,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="60" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
@@ -952,12 +952,14 @@
       <c r="J2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="4"/>
+      <c r="K2" s="4" t="s">
+        <v>91</v>
+      </c>
       <c r="L2" s="4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
@@ -988,12 +990,14 @@
       <c r="J3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="4"/>
+      <c r="K3" s="4" t="s">
+        <v>91</v>
+      </c>
       <c r="L3" s="4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>51</v>
       </c>
@@ -1027,7 +1031,7 @@
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
     </row>
-    <row r="5" spans="1:12" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>59</v>
       </c>
@@ -1063,7 +1067,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>64</v>
       </c>
@@ -1099,7 +1103,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>70</v>
       </c>
@@ -1135,7 +1139,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="60" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>74</v>
       </c>
@@ -1171,7 +1175,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="30" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>77</v>
       </c>
@@ -1202,10 +1206,12 @@
       <c r="J9" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="K9" s="4"/>
+      <c r="K9" s="4" t="s">
+        <v>91</v>
+      </c>
       <c r="L9" s="4"/>
     </row>
-    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>80</v>
       </c>
@@ -1236,12 +1242,14 @@
       <c r="J10" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="K10" s="4"/>
+      <c r="K10" s="4" t="s">
+        <v>91</v>
+      </c>
       <c r="L10" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="30" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>84</v>
       </c>
@@ -1277,7 +1285,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="60" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>94</v>
       </c>
@@ -1313,7 +1321,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="75" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>100</v>
       </c>
@@ -1349,7 +1357,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>108</v>
       </c>
@@ -1381,7 +1389,7 @@
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
     </row>
-    <row r="15" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>109</v>
       </c>
@@ -1413,7 +1421,7 @@
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
     </row>
-    <row r="16" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="60" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>110</v>
       </c>
@@ -1445,7 +1453,7 @@
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
     </row>
-    <row r="17" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>117</v>
       </c>
@@ -1481,7 +1489,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>122</v>
       </c>
@@ -1517,7 +1525,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>126</v>
       </c>
@@ -1553,7 +1561,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="45" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>131</v>
       </c>
@@ -1599,83 +1607,83 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A16"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>41</v>
       </c>

</xml_diff>

<commit_message>
SCRUM-84: Fix API product and cart validation
</commit_message>
<xml_diff>
--- a/Docs/QA-Testing/Bug_Report.xlsx
+++ b/Docs/QA-Testing/Bug_Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KiemChungPhanMem\Docs\QA-Testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KCPM - NAM3\Online-Store\Docs\QA-Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6113BAF-0A42-45A3-8D05-F988930F440B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798172ED-BA51-4339-9687-F00403ECDA55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="173">
   <si>
     <t>Bug ID</t>
   </si>
@@ -1569,7 +1569,9 @@
       <c r="I17" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="J17" s="3"/>
+      <c r="J17" s="8" t="s">
+        <v>89</v>
+      </c>
       <c r="K17" s="3" t="s">
         <v>119</v>
       </c>
@@ -1602,7 +1604,9 @@
       <c r="I18" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="J18" s="3"/>
+      <c r="J18" s="8" t="s">
+        <v>89</v>
+      </c>
       <c r="K18" s="3" t="s">
         <v>119</v>
       </c>
@@ -1635,7 +1639,9 @@
       <c r="I19" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="J19" s="3"/>
+      <c r="J19" s="8" t="s">
+        <v>89</v>
+      </c>
       <c r="K19" s="3" t="s">
         <v>128</v>
       </c>
@@ -1668,7 +1674,9 @@
       <c r="I20" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="J20" s="3"/>
+      <c r="J20" s="8" t="s">
+        <v>89</v>
+      </c>
       <c r="K20" s="3" t="s">
         <v>133</v>
       </c>
@@ -1701,7 +1709,9 @@
       <c r="I21" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="J21" s="3"/>
+      <c r="J21" s="8" t="s">
+        <v>89</v>
+      </c>
       <c r="K21" s="3" t="s">
         <v>151</v>
       </c>

</xml_diff>

<commit_message>
Doc sync round 1 – 12/09
</commit_message>
<xml_diff>
--- a/Docs/QA-Testing/Bug_Report.xlsx
+++ b/Docs/QA-Testing/Bug_Report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KiemChungPhanMem\Docs\QA-Testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Downloads/Online-Store/Docs/QA-Testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A513519-7E12-42FA-B3CF-B7F3F75DFC03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9A1D03-1648-2642-9CF1-DD95BD4AB7F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="173">
   <si>
     <t>Bug ID</t>
   </si>
@@ -65,6 +65,9 @@
     <t>TC_FE_EMP_03</t>
   </si>
   <si>
+    <t>Lưu thành công, giá âm được chấp nhận</t>
+  </si>
+  <si>
     <t>Cao</t>
   </si>
   <si>
@@ -149,6 +152,9 @@
     <t>Không cho lưu, hiện lỗi validate</t>
   </si>
   <si>
+    <t>Root cause: ProductInfo.productPrice không có @Min/@Positive. Xác nhận thêm qua CodeceptJS TC_FE_MGR_03</t>
+  </si>
+  <si>
     <t>[Product] Sửa sản phẩm cho phép nhập giá âm (Role Manager)</t>
   </si>
   <si>
@@ -158,6 +164,12 @@
     <t>Không cho lưu</t>
   </si>
   <si>
+    <t>Lưu thành công</t>
+  </si>
+  <si>
+    <t>Cùng root cause SCRUM-43</t>
+  </si>
+  <si>
     <t>SCRUM-45</t>
   </si>
   <si>
@@ -176,6 +188,9 @@
     <t>Hiện lỗi “Email/Password is required”, nút Sign In disabled</t>
   </si>
   <si>
+    <t>Nút vẫn enable / thông báo sai</t>
+  </si>
+  <si>
     <t>Thành</t>
   </si>
   <si>
@@ -266,7 +281,19 @@
     <t>Quan sát cột Status/Action</t>
   </si>
   <si>
+    <t>Viết đúng “Orders”, “Finished”, “Canceled”</t>
+  </si>
+  <si>
+    <t>Hiện “Oders”, “Cenceled” (typo)</t>
+  </si>
+  <si>
+    <t>CodeceptJS cũng bắt được “Cenceled”</t>
+  </si>
+  <si>
     <t>Thùy</t>
+  </si>
+  <si>
+    <t>TC_FE_EMP_09, TC_FE_MRG_09</t>
   </si>
   <si>
     <t>[API][Security] Hệ thống cho phép đăng ký với role tùy ý (Privilege Escalation)</t>
@@ -313,6 +340,9 @@
     <t>Trả về 500 Internal Server Error + message "Status is not correct"</t>
   </si>
   <si>
+    <t>Phát hiện từ State Transition Testing. Hệ thống có chặn nhưng xử lý exception sai.</t>
+  </si>
+  <si>
     <t>[API][Order] Invalid status transition trả về 500 thay vì 4xx</t>
   </si>
   <si>
@@ -355,6 +385,9 @@
     <t>Xem Jira SCRUM-69</t>
   </si>
   <si>
+    <t>Tách từ nhóm SCRUM-61 cũ</t>
+  </si>
+  <si>
     <t>SCRUM-70</t>
   </si>
   <si>
@@ -379,6 +412,9 @@
     <t>Xem Jira SCRUM-71</t>
   </si>
   <si>
+    <t>Thay các dòng SCRUM-61 mô tả dài</t>
+  </si>
+  <si>
     <t>SCRUM-72</t>
   </si>
   <si>
@@ -391,6 +427,9 @@
     <t>Xem Jira SCRUM-72</t>
   </si>
   <si>
+    <t>Tách khỏi SCRUM-48 (chỉ quantity)</t>
+  </si>
+  <si>
     <t>TC-REG-ROB-01</t>
   </si>
   <si>
@@ -442,6 +481,9 @@
     <t>400 Bad Request + message “Cart is empty”</t>
   </si>
   <si>
+    <t>Đã xác nhận cart rỗng bằng GET /cart trước khi gọi checkout lần 2. CartService.checkout() thiếu validate empty cart.</t>
+  </si>
+  <si>
     <t>SCRUM-79</t>
   </si>
   <si>
@@ -487,6 +529,9 @@
     <t>Subtotal = $40.00, Total = $40.00</t>
   </si>
   <si>
+    <t>Subtotal = $40,160.00, Total = $40,160.00</t>
+  </si>
+  <si>
     <t>Thêm quantity = 2 nhưng tính tiền sai rất lớn. Phát hiện từ CodeceptJS TC_FE_CUS_CART_01</t>
   </si>
   <si>
@@ -496,79 +541,10 @@
     <t>Backend trả 400 + FE hiện message “Price must be greater than 0”</t>
   </si>
   <si>
-    <t>Fixed: @Size(min=3,max=30) ProductInfo + @Valid create/edit</t>
-  </si>
-  <si>
-    <t>Fixed: @Size(min=3,max=100) productName</t>
-  </si>
-  <si>
-    <t>Fixed: @Size(max=200) productDescription</t>
-  </si>
-  <si>
-    <t>Fixed: @Size ItemForm.productId + @Valid addToCart</t>
-  </si>
-  <si>
-    <t>Fixed: CartServiceImpl throw CART_EMPTY; empty checkout = 400</t>
-  </si>
-  <si>
-    <t>401 Bad Request</t>
-  </si>
-  <si>
-    <t>402 Bad Request</t>
-  </si>
-  <si>
-    <t>403 Bad Request</t>
-  </si>
-  <si>
-    <t>404 Bad Request</t>
-  </si>
-  <si>
-    <t>API: 400 (không lưu giá âm). FE Employee: không hiện message lỗi</t>
-  </si>
-  <si>
-    <t>API: 400. FE Manager: không hiện message</t>
-  </si>
-  <si>
-    <t>API đã có @Positive. Phần còn lại = FE không bind lỗi → xem SCRUM-81. Codecept EMP_03 vẫn FAIL.</t>
-  </si>
-  <si>
-    <t>Cùng root FE với SCRUM-81. Có thể Done phần API; FE theo dõi SCRUM-81.</t>
-  </si>
-  <si>
-    <t>400 “Cart is empty”</t>
-  </si>
-  <si>
-    <t>Fixed @ControllerAdvice</t>
-  </si>
-  <si>
-    <t>PASS (retest Codecept CART_01)</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>PASS (retest Codecept CHK_01)</t>
-  </si>
-  <si>
-    <t>Email/Password trống → hiện “Email is required” / “Password is required”, nút Sign In disabled</t>
-  </si>
-  <si>
-    <t>Fixed  12/09. Đổi [hidden] → *ngIf, sửa text Password</t>
-  </si>
-  <si>
-    <t>Fixed 12/09. Sửa enum Cenceled → Canceled</t>
-  </si>
-  <si>
-    <t>Status hiển thị đúng “Canceled”</t>
-  </si>
-  <si>
-    <t>Viết đúng “Canceled”</t>
-  </si>
-  <si>
-    <t>Fixed 12/09. Bind error 400, hiện alert dưới ô Price</t>
-  </si>
-  <si>
-    <t>Backend 400 + FE hiện “Price must be greater than 0”</t>
+    <t>Backend trả 400 đúng, nhưng FE không hiện bất kỳ message lỗi nào</t>
+  </si>
+  <si>
+    <t>API đã fix (SCRUM-43/44). FE không hiển thị lỗi từ response. Phát hiện từ CodeceptJS TC_FE_MGR_03 + Network tab</t>
   </si>
 </sst>
 </file>
@@ -1004,22 +980,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K24"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.88671875" customWidth="1"/>
-    <col min="2" max="2" width="30.44140625" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.5" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="22.44140625" customWidth="1"/>
+    <col min="4" max="4" width="22.5" customWidth="1"/>
     <col min="5" max="5" width="36" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
-    <col min="8" max="8" width="15.109375" customWidth="1"/>
+    <col min="8" max="8" width="15.1640625" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="39.44140625" customWidth="1"/>
+    <col min="11" max="11" width="39.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1054,12 +1030,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>12</v>
@@ -1068,252 +1044,250 @@
         <v>13</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>165</v>
+        <v>14</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="45" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>166</v>
+        <v>47</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="60" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>45</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>49</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>174</v>
+        <v>55</v>
       </c>
       <c r="H4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="54" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="I5" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K5" s="3" t="s">
+      <c r="D6" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="J6" s="5" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>51</v>
-      </c>
       <c r="K6" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F7" s="3">
         <v>400</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="60" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="68" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="I8" s="5" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.3">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F9" s="3">
         <v>400</v>
@@ -1322,533 +1296,529 @@
         <v>500</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F10" s="3">
         <v>400</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="J10" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="K10" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="K10" s="3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="30" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
-        <v>77</v>
+    </row>
+    <row r="11" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>82</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>172</v>
+        <v>90</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>178</v>
+        <v>86</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>177</v>
+        <v>87</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="J11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="68" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K11" s="3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="60" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="I12" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="75" x14ac:dyDescent="0.3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="60" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="68" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A15" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="45" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="D15" s="3" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A16" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J15" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="60" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="D16" s="3" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="F17" s="3">
+        <v>400</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F18" s="3">
+        <v>400</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="F19" s="3">
+        <v>400</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="F20" s="3">
+        <v>400</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="102" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="68" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="H22" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J16" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="45" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C17" s="3" t="s">
+      <c r="I22" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="119" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="85" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="H24" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="K17" s="3" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="45" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J18" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="45" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J19" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="45" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I20" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J20" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="K20" s="3" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="90" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="K21" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="60" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I22" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J22" s="3" t="s">
+      <c r="I24" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="K24" s="3" t="s">
         <v>172</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="120" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I23" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J23" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K23" s="3" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="75" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I24" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J24" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -1861,85 +1831,85 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A16"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>